<commit_message>
rm MS from organization.contact and add MS to telecom mailbox mss aaa7a6bd6f8d534aa35f5fe88916bb4038f69df0
</commit_message>
<xml_diff>
--- a/ig/nr-change-mss-Org/StructureDefinition-as-dp-organization.xlsx
+++ b/ig/nr-change-mss-Org/StructureDefinition-as-dp-organization.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-06-15T11:25:47+00:00</t>
+    <t>2023-06-15T14:56:56+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1595,13 +1595,13 @@
 </t>
   </si>
   <si>
-    <t>Point de contact.</t>
+    <t>Contact for the organization for a certain purpose</t>
   </si>
   <si>
     <t>Contact for the organization for a certain purpose.</t>
   </si>
   <si>
-    <t>Personne ou service agissant comme point de contact auprès d'une autre personne ou d'un autre service.</t>
+    <t>Where multiple contacts for the same purpose are provided there is a standard extension that can be used to determine which one is the preferred contact to use.</t>
   </si>
   <si>
     <t>Need to keep track of assigned contact points within bigger organization.</t>
@@ -11929,7 +11929,7 @@
         <v>36</v>
       </c>
       <c r="H97" t="s" s="2">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="I97" t="s" s="2">
         <v>35</v>
@@ -12851,7 +12851,7 @@
         <v>36</v>
       </c>
       <c r="H106" t="s" s="2">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="I106" t="s" s="2">
         <v>35</v>

</xml_diff>

<commit_message>
remove telecom.period.id and telecom.period.start from dp organization bb1541998ed2c92f58b2e2bd463267486aac1af1
</commit_message>
<xml_diff>
--- a/ig/nr-change-mss-Org/StructureDefinition-as-dp-organization.xlsx
+++ b/ig/nr-change-mss-Org/StructureDefinition-as-dp-organization.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AJ$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AJ$102</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3719" uniqueCount="538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3333" uniqueCount="493">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-06-15T15:17:55+00:00</t>
+    <t>2023-06-15T15:23:36+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1312,145 +1312,6 @@
   <si>
     <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
 cpt-2:A system is required if a value is provided. {value.empty() or system.exists()}org-3:The telecom of an organization can never be of use 'home' {where(use = 'home').empty()}</t>
-  </si>
-  <si>
-    <t>Organization.telecom.id</t>
-  </si>
-  <si>
-    <t>Organization.telecom.extension</t>
-  </si>
-  <si>
-    <t>Organization.telecom.extension:emailType</t>
-  </si>
-  <si>
-    <t>emailType</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extension {http://interopsante.org/fhir/StructureDefinition/FrContactPointEmailType}
-</t>
-  </si>
-  <si>
-    <t>Type of email | type de messagerie électronique</t>
-  </si>
-  <si>
-    <t>Organization.telecom.system</t>
-  </si>
-  <si>
-    <t>phone | fax | email | pager | url | sms | other</t>
-  </si>
-  <si>
-    <t>Telecommunications form for contact point - what communications system is required to make use of the contact.</t>
-  </si>
-  <si>
-    <t>https://www.hl7.org/fhir/valueset-contact-point-system.html</t>
-  </si>
-  <si>
-    <t>Telecommunications form for contact point.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/contact-point-system</t>
-  </si>
-  <si>
-    <t>ContactPoint.system</t>
-  </si>
-  <si>
-    <t>ele-1
-cpt-2</t>
-  </si>
-  <si>
-    <t>Organization.telecom.value</t>
-  </si>
-  <si>
-    <t>The actual contact point details</t>
-  </si>
-  <si>
-    <t>The actual contact point details, in a form that is meaningful to the designated communication system (i.e. phone number or email address).</t>
-  </si>
-  <si>
-    <t>Additional text data such as phone extension numbers, or notes about use of the contact are sometimes included in the value.</t>
-  </si>
-  <si>
-    <t>Need to support legacy numbers that are not in a tightly controlled format.</t>
-  </si>
-  <si>
-    <t>ContactPoint.value</t>
-  </si>
-  <si>
-    <t>Organization.telecom.use</t>
-  </si>
-  <si>
-    <t>home | work | temp | old | mobile - purpose of this contact point</t>
-  </si>
-  <si>
-    <t>Identifies the purpose for the contact point.</t>
-  </si>
-  <si>
-    <t>« old » si les coordonnées de structure ont une date de fin</t>
-  </si>
-  <si>
-    <t>Need to track the way a person uses this contact, so a user can choose which is appropriate for their purpose.</t>
-  </si>
-  <si>
-    <t>Use of contact point.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/contact-point-use</t>
-  </si>
-  <si>
-    <t>ContactPoint.use</t>
-  </si>
-  <si>
-    <t>Organization.telecom.rank</t>
-  </si>
-  <si>
-    <t xml:space="preserve">positiveInt
-</t>
-  </si>
-  <si>
-    <t>Specify preferred order of use (1 = highest)</t>
-  </si>
-  <si>
-    <t>Specifies a preferred order in which to use a set of contacts. ContactPoints with lower rank values are more preferred than those with higher rank values.</t>
-  </si>
-  <si>
-    <t>Note that rank does not necessarily follow the order in which the contacts are represented in the instance.</t>
-  </si>
-  <si>
-    <t>ContactPoint.rank</t>
-  </si>
-  <si>
-    <t>Organization.telecom.period</t>
-  </si>
-  <si>
-    <t>Time period when the contact point was/is in use</t>
-  </si>
-  <si>
-    <t>Time period when the contact point was/is in use.</t>
-  </si>
-  <si>
-    <t>A Period specifies a range of time; the context of use will specify whether the entire range applies (e.g. "the patient was an inpatient of the hospital for this time range") or one value from the range applies (e.g. "give to the patient between these two times").
-Period is not used for a duration (a measure of elapsed time). See [Duration](http://hl7.org/fhir/R4/datatypes.html#Duration).</t>
-  </si>
-  <si>
-    <t>ContactPoint.period</t>
-  </si>
-  <si>
-    <t>Organization.telecom.period.id</t>
-  </si>
-  <si>
-    <t>Organization.telecom.period.extension</t>
-  </si>
-  <si>
-    <t>Organization.telecom.period.start</t>
-  </si>
-  <si>
-    <t>Starting time with inclusive boundary</t>
-  </si>
-  <si>
-    <t>Organization.telecom.period.end</t>
-  </si>
-  <si>
-    <t>End time with inclusive boundary, if not ongoing</t>
   </si>
   <si>
     <t>Organization.telecom:mailbox-mss</t>
@@ -2018,7 +1879,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AJ114"/>
+  <dimension ref="A1:AJ102"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="63.859375" customWidth="true" bestFit="true"/>
@@ -10682,9 +10543,11 @@
         <v>412</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>412</v>
-      </c>
-      <c r="C85" s="2"/>
+        <v>403</v>
+      </c>
+      <c r="C85" t="s" s="2">
+        <v>413</v>
+      </c>
       <c r="D85" t="s" s="2">
         <v>35</v>
       </c>
@@ -10693,10 +10556,10 @@
         <v>36</v>
       </c>
       <c r="G85" t="s" s="2">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="H85" t="s" s="2">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="I85" t="s" s="2">
         <v>35</v>
@@ -10705,16 +10568,20 @@
         <v>35</v>
       </c>
       <c r="K85" t="s" s="2">
-        <v>56</v>
+        <v>414</v>
       </c>
       <c r="L85" t="s" s="2">
-        <v>57</v>
+        <v>415</v>
       </c>
       <c r="M85" t="s" s="2">
-        <v>58</v>
-      </c>
-      <c r="N85" s="2"/>
-      <c r="O85" s="2"/>
+        <v>406</v>
+      </c>
+      <c r="N85" t="s" s="2">
+        <v>407</v>
+      </c>
+      <c r="O85" t="s" s="2">
+        <v>408</v>
+      </c>
       <c r="P85" t="s" s="2">
         <v>35</v>
       </c>
@@ -10762,31 +10629,31 @@
         <v>35</v>
       </c>
       <c r="AF85" t="s" s="2">
-        <v>59</v>
+        <v>403</v>
       </c>
       <c r="AG85" t="s" s="2">
         <v>36</v>
       </c>
       <c r="AH85" t="s" s="2">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="AI85" t="s" s="2">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="AJ85" t="s" s="2">
-        <v>35</v>
+        <v>411</v>
       </c>
     </row>
     <row r="86" hidden="true">
       <c r="A86" t="s" s="2">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="E86" s="2"/>
       <c r="F86" t="s" s="2">
@@ -10796,7 +10663,7 @@
         <v>37</v>
       </c>
       <c r="H86" t="s" s="2">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="I86" t="s" s="2">
         <v>35</v>
@@ -10805,18 +10672,20 @@
         <v>35</v>
       </c>
       <c r="K86" t="s" s="2">
-        <v>62</v>
+        <v>417</v>
       </c>
       <c r="L86" t="s" s="2">
-        <v>63</v>
+        <v>418</v>
       </c>
       <c r="M86" t="s" s="2">
-        <v>64</v>
+        <v>419</v>
       </c>
       <c r="N86" t="s" s="2">
-        <v>65</v>
-      </c>
-      <c r="O86" s="2"/>
+        <v>420</v>
+      </c>
+      <c r="O86" t="s" s="2">
+        <v>421</v>
+      </c>
       <c r="P86" t="s" s="2">
         <v>35</v>
       </c>
@@ -10852,19 +10721,19 @@
         <v>35</v>
       </c>
       <c r="AB86" t="s" s="2">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="AC86" t="s" s="2">
-        <v>67</v>
+        <v>35</v>
       </c>
       <c r="AD86" t="s" s="2">
         <v>35</v>
       </c>
       <c r="AE86" t="s" s="2">
-        <v>68</v>
+        <v>35</v>
       </c>
       <c r="AF86" t="s" s="2">
-        <v>69</v>
+        <v>416</v>
       </c>
       <c r="AG86" t="s" s="2">
         <v>36</v>
@@ -10876,21 +10745,19 @@
         <v>54</v>
       </c>
       <c r="AJ86" t="s" s="2">
-        <v>70</v>
+        <v>422</v>
       </c>
     </row>
     <row r="87" hidden="true">
       <c r="A87" t="s" s="2">
-        <v>414</v>
+        <v>423</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>413</v>
-      </c>
-      <c r="C87" t="s" s="2">
-        <v>415</v>
-      </c>
+        <v>423</v>
+      </c>
+      <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="E87" s="2"/>
       <c r="F87" t="s" s="2">
@@ -10906,21 +10773,23 @@
         <v>35</v>
       </c>
       <c r="J87" t="s" s="2">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="K87" t="s" s="2">
-        <v>416</v>
+        <v>424</v>
       </c>
       <c r="L87" t="s" s="2">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="M87" t="s" s="2">
-        <v>153</v>
+        <v>426</v>
       </c>
       <c r="N87" t="s" s="2">
-        <v>65</v>
-      </c>
-      <c r="O87" s="2"/>
+        <v>427</v>
+      </c>
+      <c r="O87" t="s" s="2">
+        <v>428</v>
+      </c>
       <c r="P87" t="s" s="2">
         <v>35</v>
       </c>
@@ -10968,27 +10837,27 @@
         <v>35</v>
       </c>
       <c r="AF87" t="s" s="2">
-        <v>69</v>
+        <v>423</v>
       </c>
       <c r="AG87" t="s" s="2">
         <v>36</v>
       </c>
       <c r="AH87" t="s" s="2">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="AI87" t="s" s="2">
         <v>54</v>
       </c>
       <c r="AJ87" t="s" s="2">
-        <v>70</v>
+        <v>267</v>
       </c>
     </row>
     <row r="88" hidden="true">
       <c r="A88" t="s" s="2">
-        <v>418</v>
+        <v>429</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>418</v>
+        <v>429</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -10996,7 +10865,7 @@
       </c>
       <c r="E88" s="2"/>
       <c r="F88" t="s" s="2">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="G88" t="s" s="2">
         <v>42</v>
@@ -11008,20 +10877,18 @@
         <v>35</v>
       </c>
       <c r="J88" t="s" s="2">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="K88" t="s" s="2">
-        <v>123</v>
+        <v>56</v>
       </c>
       <c r="L88" t="s" s="2">
-        <v>419</v>
+        <v>57</v>
       </c>
       <c r="M88" t="s" s="2">
-        <v>420</v>
-      </c>
-      <c r="N88" t="s" s="2">
-        <v>421</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="N88" s="2"/>
       <c r="O88" s="2"/>
       <c r="P88" t="s" s="2">
         <v>35</v>
@@ -11046,13 +10913,13 @@
         <v>35</v>
       </c>
       <c r="X88" t="s" s="2">
-        <v>228</v>
+        <v>35</v>
       </c>
       <c r="Y88" t="s" s="2">
-        <v>422</v>
+        <v>35</v>
       </c>
       <c r="Z88" t="s" s="2">
-        <v>423</v>
+        <v>35</v>
       </c>
       <c r="AA88" t="s" s="2">
         <v>35</v>
@@ -11070,7 +10937,7 @@
         <v>35</v>
       </c>
       <c r="AF88" t="s" s="2">
-        <v>424</v>
+        <v>59</v>
       </c>
       <c r="AG88" t="s" s="2">
         <v>36</v>
@@ -11079,29 +10946,29 @@
         <v>42</v>
       </c>
       <c r="AI88" t="s" s="2">
-        <v>425</v>
+        <v>35</v>
       </c>
       <c r="AJ88" t="s" s="2">
-        <v>81</v>
+        <v>35</v>
       </c>
     </row>
     <row r="89" hidden="true">
       <c r="A89" t="s" s="2">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="E89" s="2"/>
       <c r="F89" t="s" s="2">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="G89" t="s" s="2">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="H89" t="s" s="2">
         <v>35</v>
@@ -11110,23 +10977,21 @@
         <v>35</v>
       </c>
       <c r="J89" t="s" s="2">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="K89" t="s" s="2">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="L89" t="s" s="2">
-        <v>427</v>
+        <v>63</v>
       </c>
       <c r="M89" t="s" s="2">
-        <v>428</v>
+        <v>64</v>
       </c>
       <c r="N89" t="s" s="2">
-        <v>429</v>
-      </c>
-      <c r="O89" t="s" s="2">
-        <v>430</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="O89" s="2"/>
       <c r="P89" t="s" s="2">
         <v>35</v>
       </c>
@@ -11162,39 +11027,39 @@
         <v>35</v>
       </c>
       <c r="AB89" t="s" s="2">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="AC89" t="s" s="2">
-        <v>35</v>
+        <v>67</v>
       </c>
       <c r="AD89" t="s" s="2">
         <v>35</v>
       </c>
       <c r="AE89" t="s" s="2">
-        <v>35</v>
+        <v>68</v>
       </c>
       <c r="AF89" t="s" s="2">
-        <v>431</v>
+        <v>69</v>
       </c>
       <c r="AG89" t="s" s="2">
         <v>36</v>
       </c>
       <c r="AH89" t="s" s="2">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="AI89" t="s" s="2">
         <v>54</v>
       </c>
       <c r="AJ89" t="s" s="2">
-        <v>81</v>
+        <v>70</v>
       </c>
     </row>
     <row r="90" hidden="true">
       <c r="A90" t="s" s="2">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -11211,26 +11076,24 @@
         <v>35</v>
       </c>
       <c r="I90" t="s" s="2">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="J90" t="s" s="2">
         <v>43</v>
       </c>
       <c r="K90" t="s" s="2">
-        <v>123</v>
+        <v>56</v>
       </c>
       <c r="L90" t="s" s="2">
+        <v>432</v>
+      </c>
+      <c r="M90" t="s" s="2">
         <v>433</v>
       </c>
-      <c r="M90" t="s" s="2">
+      <c r="N90" t="s" s="2">
         <v>434</v>
       </c>
-      <c r="N90" t="s" s="2">
-        <v>435</v>
-      </c>
-      <c r="O90" t="s" s="2">
-        <v>436</v>
-      </c>
+      <c r="O90" s="2"/>
       <c r="P90" t="s" s="2">
         <v>35</v>
       </c>
@@ -11254,13 +11117,13 @@
         <v>35</v>
       </c>
       <c r="X90" t="s" s="2">
-        <v>228</v>
+        <v>35</v>
       </c>
       <c r="Y90" t="s" s="2">
-        <v>437</v>
+        <v>35</v>
       </c>
       <c r="Z90" t="s" s="2">
-        <v>438</v>
+        <v>35</v>
       </c>
       <c r="AA90" t="s" s="2">
         <v>35</v>
@@ -11278,7 +11141,7 @@
         <v>35</v>
       </c>
       <c r="AF90" t="s" s="2">
-        <v>439</v>
+        <v>435</v>
       </c>
       <c r="AG90" t="s" s="2">
         <v>36</v>
@@ -11287,7 +11150,7 @@
         <v>42</v>
       </c>
       <c r="AI90" t="s" s="2">
-        <v>54</v>
+        <v>436</v>
       </c>
       <c r="AJ90" t="s" s="2">
         <v>81</v>
@@ -11295,10 +11158,10 @@
     </row>
     <row r="91" hidden="true">
       <c r="A91" t="s" s="2">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -11321,16 +11184,16 @@
         <v>43</v>
       </c>
       <c r="K91" t="s" s="2">
-        <v>441</v>
+        <v>89</v>
       </c>
       <c r="L91" t="s" s="2">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="M91" t="s" s="2">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="N91" t="s" s="2">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="O91" s="2"/>
       <c r="P91" t="s" s="2">
@@ -11356,13 +11219,13 @@
         <v>35</v>
       </c>
       <c r="X91" t="s" s="2">
-        <v>35</v>
+        <v>105</v>
       </c>
       <c r="Y91" t="s" s="2">
-        <v>35</v>
+        <v>441</v>
       </c>
       <c r="Z91" t="s" s="2">
-        <v>35</v>
+        <v>287</v>
       </c>
       <c r="AA91" t="s" s="2">
         <v>35</v>
@@ -11380,7 +11243,7 @@
         <v>35</v>
       </c>
       <c r="AF91" t="s" s="2">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="AG91" t="s" s="2">
         <v>36</v>
@@ -11397,10 +11260,10 @@
     </row>
     <row r="92" hidden="true">
       <c r="A92" t="s" s="2">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -11423,16 +11286,16 @@
         <v>43</v>
       </c>
       <c r="K92" t="s" s="2">
-        <v>175</v>
+        <v>215</v>
       </c>
       <c r="L92" t="s" s="2">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="M92" t="s" s="2">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="N92" t="s" s="2">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="O92" s="2"/>
       <c r="P92" t="s" s="2">
@@ -11482,7 +11345,7 @@
         <v>35</v>
       </c>
       <c r="AF92" t="s" s="2">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="AG92" t="s" s="2">
         <v>36</v>
@@ -11494,15 +11357,15 @@
         <v>54</v>
       </c>
       <c r="AJ92" t="s" s="2">
-        <v>260</v>
+        <v>81</v>
       </c>
     </row>
     <row r="93" hidden="true">
       <c r="A93" t="s" s="2">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -11513,7 +11376,7 @@
         <v>36</v>
       </c>
       <c r="G93" t="s" s="2">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="H93" t="s" s="2">
         <v>35</v>
@@ -11522,18 +11385,20 @@
         <v>35</v>
       </c>
       <c r="J93" t="s" s="2">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="K93" t="s" s="2">
         <v>56</v>
       </c>
       <c r="L93" t="s" s="2">
-        <v>57</v>
+        <v>449</v>
       </c>
       <c r="M93" t="s" s="2">
-        <v>58</v>
-      </c>
-      <c r="N93" s="2"/>
+        <v>450</v>
+      </c>
+      <c r="N93" t="s" s="2">
+        <v>451</v>
+      </c>
       <c r="O93" s="2"/>
       <c r="P93" t="s" s="2">
         <v>35</v>
@@ -11582,7 +11447,7 @@
         <v>35</v>
       </c>
       <c r="AF93" t="s" s="2">
-        <v>59</v>
+        <v>452</v>
       </c>
       <c r="AG93" t="s" s="2">
         <v>36</v>
@@ -11591,29 +11456,29 @@
         <v>42</v>
       </c>
       <c r="AI93" t="s" s="2">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="AJ93" t="s" s="2">
-        <v>35</v>
+        <v>81</v>
       </c>
     </row>
     <row r="94" hidden="true">
       <c r="A94" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="E94" s="2"/>
       <c r="F94" t="s" s="2">
         <v>36</v>
       </c>
       <c r="G94" t="s" s="2">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H94" t="s" s="2">
         <v>35</v>
@@ -11625,18 +11490,20 @@
         <v>35</v>
       </c>
       <c r="K94" t="s" s="2">
-        <v>62</v>
+        <v>454</v>
       </c>
       <c r="L94" t="s" s="2">
-        <v>63</v>
+        <v>455</v>
       </c>
       <c r="M94" t="s" s="2">
-        <v>64</v>
+        <v>456</v>
       </c>
       <c r="N94" t="s" s="2">
-        <v>65</v>
-      </c>
-      <c r="O94" s="2"/>
+        <v>457</v>
+      </c>
+      <c r="O94" t="s" s="2">
+        <v>458</v>
+      </c>
       <c r="P94" t="s" s="2">
         <v>35</v>
       </c>
@@ -11672,19 +11539,19 @@
         <v>35</v>
       </c>
       <c r="AB94" t="s" s="2">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="AC94" t="s" s="2">
-        <v>67</v>
+        <v>35</v>
       </c>
       <c r="AD94" t="s" s="2">
         <v>35</v>
       </c>
       <c r="AE94" t="s" s="2">
-        <v>68</v>
+        <v>35</v>
       </c>
       <c r="AF94" t="s" s="2">
-        <v>69</v>
+        <v>453</v>
       </c>
       <c r="AG94" t="s" s="2">
         <v>36</v>
@@ -11696,15 +11563,15 @@
         <v>54</v>
       </c>
       <c r="AJ94" t="s" s="2">
-        <v>70</v>
+        <v>81</v>
       </c>
     </row>
     <row r="95" hidden="true">
       <c r="A95" t="s" s="2">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -11715,7 +11582,7 @@
         <v>36</v>
       </c>
       <c r="G95" t="s" s="2">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="H95" t="s" s="2">
         <v>35</v>
@@ -11724,20 +11591,18 @@
         <v>35</v>
       </c>
       <c r="J95" t="s" s="2">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="K95" t="s" s="2">
-        <v>185</v>
+        <v>56</v>
       </c>
       <c r="L95" t="s" s="2">
-        <v>454</v>
+        <v>57</v>
       </c>
       <c r="M95" t="s" s="2">
-        <v>187</v>
-      </c>
-      <c r="N95" t="s" s="2">
-        <v>188</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="N95" s="2"/>
       <c r="O95" s="2"/>
       <c r="P95" t="s" s="2">
         <v>35</v>
@@ -11786,7 +11651,7 @@
         <v>35</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>189</v>
+        <v>59</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>36</v>
@@ -11795,29 +11660,29 @@
         <v>42</v>
       </c>
       <c r="AI95" t="s" s="2">
-        <v>190</v>
+        <v>35</v>
       </c>
       <c r="AJ95" t="s" s="2">
-        <v>81</v>
+        <v>35</v>
       </c>
     </row>
     <row r="96" hidden="true">
       <c r="A96" t="s" s="2">
-        <v>455</v>
+        <v>460</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>455</v>
+        <v>460</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="E96" s="2"/>
       <c r="F96" t="s" s="2">
         <v>36</v>
       </c>
       <c r="G96" t="s" s="2">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="H96" t="s" s="2">
         <v>35</v>
@@ -11826,27 +11691,25 @@
         <v>35</v>
       </c>
       <c r="J96" t="s" s="2">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="K96" t="s" s="2">
-        <v>185</v>
+        <v>62</v>
       </c>
       <c r="L96" t="s" s="2">
-        <v>456</v>
+        <v>63</v>
       </c>
       <c r="M96" t="s" s="2">
-        <v>194</v>
+        <v>64</v>
       </c>
       <c r="N96" t="s" s="2">
-        <v>195</v>
+        <v>65</v>
       </c>
       <c r="O96" s="2"/>
       <c r="P96" t="s" s="2">
         <v>35</v>
       </c>
-      <c r="Q96" t="s" s="2">
-        <v>196</v>
-      </c>
+      <c r="Q96" s="2"/>
       <c r="R96" t="s" s="2">
         <v>35</v>
       </c>
@@ -11878,76 +11741,74 @@
         <v>35</v>
       </c>
       <c r="AB96" t="s" s="2">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="AC96" t="s" s="2">
-        <v>35</v>
+        <v>67</v>
       </c>
       <c r="AD96" t="s" s="2">
         <v>35</v>
       </c>
       <c r="AE96" t="s" s="2">
-        <v>35</v>
+        <v>68</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>197</v>
+        <v>69</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>36</v>
       </c>
       <c r="AH96" t="s" s="2">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="AI96" t="s" s="2">
-        <v>190</v>
+        <v>54</v>
       </c>
       <c r="AJ96" t="s" s="2">
-        <v>81</v>
+        <v>70</v>
       </c>
     </row>
     <row r="97" hidden="true">
       <c r="A97" t="s" s="2">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>403</v>
-      </c>
-      <c r="C97" t="s" s="2">
-        <v>458</v>
-      </c>
+        <v>461</v>
+      </c>
+      <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
-        <v>35</v>
+        <v>462</v>
       </c>
       <c r="E97" s="2"/>
       <c r="F97" t="s" s="2">
         <v>36</v>
       </c>
       <c r="G97" t="s" s="2">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H97" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="I97" t="s" s="2">
         <v>43</v>
       </c>
-      <c r="I97" t="s" s="2">
-        <v>35</v>
-      </c>
       <c r="J97" t="s" s="2">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="K97" t="s" s="2">
-        <v>459</v>
+        <v>62</v>
       </c>
       <c r="L97" t="s" s="2">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="M97" t="s" s="2">
-        <v>406</v>
+        <v>464</v>
       </c>
       <c r="N97" t="s" s="2">
-        <v>407</v>
+        <v>65</v>
       </c>
       <c r="O97" t="s" s="2">
-        <v>408</v>
+        <v>212</v>
       </c>
       <c r="P97" t="s" s="2">
         <v>35</v>
@@ -11996,7 +11857,7 @@
         <v>35</v>
       </c>
       <c r="AF97" t="s" s="2">
-        <v>403</v>
+        <v>465</v>
       </c>
       <c r="AG97" t="s" s="2">
         <v>36</v>
@@ -12008,15 +11869,15 @@
         <v>54</v>
       </c>
       <c r="AJ97" t="s" s="2">
-        <v>411</v>
+        <v>70</v>
       </c>
     </row>
     <row r="98" hidden="true">
       <c r="A98" t="s" s="2">
-        <v>461</v>
+        <v>466</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>461</v>
+        <v>466</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -12027,10 +11888,10 @@
         <v>36</v>
       </c>
       <c r="G98" t="s" s="2">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="H98" t="s" s="2">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="I98" t="s" s="2">
         <v>35</v>
@@ -12039,19 +11900,19 @@
         <v>35</v>
       </c>
       <c r="K98" t="s" s="2">
-        <v>462</v>
+        <v>233</v>
       </c>
       <c r="L98" t="s" s="2">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="M98" t="s" s="2">
-        <v>464</v>
+        <v>468</v>
       </c>
       <c r="N98" t="s" s="2">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="O98" t="s" s="2">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="P98" t="s" s="2">
         <v>35</v>
@@ -12076,13 +11937,13 @@
         <v>35</v>
       </c>
       <c r="X98" t="s" s="2">
-        <v>35</v>
+        <v>105</v>
       </c>
       <c r="Y98" t="s" s="2">
-        <v>35</v>
+        <v>471</v>
       </c>
       <c r="Z98" t="s" s="2">
-        <v>35</v>
+        <v>472</v>
       </c>
       <c r="AA98" t="s" s="2">
         <v>35</v>
@@ -12100,27 +11961,27 @@
         <v>35</v>
       </c>
       <c r="AF98" t="s" s="2">
-        <v>461</v>
+        <v>466</v>
       </c>
       <c r="AG98" t="s" s="2">
         <v>36</v>
       </c>
       <c r="AH98" t="s" s="2">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="AI98" t="s" s="2">
         <v>54</v>
       </c>
       <c r="AJ98" t="s" s="2">
-        <v>467</v>
+        <v>81</v>
       </c>
     </row>
     <row r="99" hidden="true">
       <c r="A99" t="s" s="2">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
@@ -12140,22 +12001,22 @@
         <v>35</v>
       </c>
       <c r="J99" t="s" s="2">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="K99" t="s" s="2">
-        <v>469</v>
+        <v>474</v>
       </c>
       <c r="L99" t="s" s="2">
-        <v>470</v>
+        <v>475</v>
       </c>
       <c r="M99" t="s" s="2">
-        <v>471</v>
+        <v>476</v>
       </c>
       <c r="N99" t="s" s="2">
-        <v>472</v>
+        <v>477</v>
       </c>
       <c r="O99" t="s" s="2">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="P99" t="s" s="2">
         <v>35</v>
@@ -12204,7 +12065,7 @@
         <v>35</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>36</v>
@@ -12216,15 +12077,15 @@
         <v>54</v>
       </c>
       <c r="AJ99" t="s" s="2">
-        <v>267</v>
+        <v>81</v>
       </c>
     </row>
     <row r="100" hidden="true">
       <c r="A100" t="s" s="2">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -12235,7 +12096,7 @@
         <v>36</v>
       </c>
       <c r="G100" t="s" s="2">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="H100" t="s" s="2">
         <v>35</v>
@@ -12247,16 +12108,18 @@
         <v>35</v>
       </c>
       <c r="K100" t="s" s="2">
-        <v>56</v>
+        <v>404</v>
       </c>
       <c r="L100" t="s" s="2">
-        <v>57</v>
+        <v>415</v>
       </c>
       <c r="M100" t="s" s="2">
-        <v>58</v>
+        <v>406</v>
       </c>
       <c r="N100" s="2"/>
-      <c r="O100" s="2"/>
+      <c r="O100" t="s" s="2">
+        <v>480</v>
+      </c>
       <c r="P100" t="s" s="2">
         <v>35</v>
       </c>
@@ -12304,38 +12167,38 @@
         <v>35</v>
       </c>
       <c r="AF100" t="s" s="2">
-        <v>59</v>
+        <v>479</v>
       </c>
       <c r="AG100" t="s" s="2">
         <v>36</v>
       </c>
       <c r="AH100" t="s" s="2">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="AI100" t="s" s="2">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="AJ100" t="s" s="2">
-        <v>35</v>
+        <v>481</v>
       </c>
     </row>
     <row r="101" hidden="true">
       <c r="A101" t="s" s="2">
-        <v>475</v>
+        <v>482</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>475</v>
+        <v>482</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="E101" s="2"/>
       <c r="F101" t="s" s="2">
         <v>36</v>
       </c>
       <c r="G101" t="s" s="2">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="H101" t="s" s="2">
         <v>35</v>
@@ -12347,18 +12210,20 @@
         <v>35</v>
       </c>
       <c r="K101" t="s" s="2">
-        <v>62</v>
+        <v>483</v>
       </c>
       <c r="L101" t="s" s="2">
-        <v>63</v>
+        <v>484</v>
       </c>
       <c r="M101" t="s" s="2">
-        <v>64</v>
+        <v>419</v>
       </c>
       <c r="N101" t="s" s="2">
-        <v>65</v>
-      </c>
-      <c r="O101" s="2"/>
+        <v>485</v>
+      </c>
+      <c r="O101" t="s" s="2">
+        <v>486</v>
+      </c>
       <c r="P101" t="s" s="2">
         <v>35</v>
       </c>
@@ -12394,39 +12259,39 @@
         <v>35</v>
       </c>
       <c r="AB101" t="s" s="2">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="AC101" t="s" s="2">
-        <v>67</v>
+        <v>35</v>
       </c>
       <c r="AD101" t="s" s="2">
         <v>35</v>
       </c>
       <c r="AE101" t="s" s="2">
-        <v>68</v>
+        <v>35</v>
       </c>
       <c r="AF101" t="s" s="2">
-        <v>69</v>
+        <v>482</v>
       </c>
       <c r="AG101" t="s" s="2">
         <v>36</v>
       </c>
       <c r="AH101" t="s" s="2">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="AI101" t="s" s="2">
         <v>54</v>
       </c>
       <c r="AJ101" t="s" s="2">
-        <v>70</v>
+        <v>81</v>
       </c>
     </row>
     <row r="102" hidden="true">
       <c r="A102" t="s" s="2">
-        <v>476</v>
+        <v>487</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>476</v>
+        <v>487</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -12437,30 +12302,32 @@
         <v>36</v>
       </c>
       <c r="G102" t="s" s="2">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="H102" t="s" s="2">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="I102" t="s" s="2">
         <v>35</v>
       </c>
       <c r="J102" t="s" s="2">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="K102" t="s" s="2">
-        <v>56</v>
+        <v>488</v>
       </c>
       <c r="L102" t="s" s="2">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="M102" t="s" s="2">
-        <v>478</v>
+        <v>490</v>
       </c>
       <c r="N102" t="s" s="2">
-        <v>479</v>
-      </c>
-      <c r="O102" s="2"/>
+        <v>491</v>
+      </c>
+      <c r="O102" t="s" s="2">
+        <v>492</v>
+      </c>
       <c r="P102" t="s" s="2">
         <v>35</v>
       </c>
@@ -12508,1257 +12375,23 @@
         <v>35</v>
       </c>
       <c r="AF102" t="s" s="2">
-        <v>480</v>
+        <v>487</v>
       </c>
       <c r="AG102" t="s" s="2">
         <v>36</v>
       </c>
       <c r="AH102" t="s" s="2">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="AI102" t="s" s="2">
-        <v>481</v>
+        <v>54</v>
       </c>
       <c r="AJ102" t="s" s="2">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="103" hidden="true">
-      <c r="A103" t="s" s="2">
-        <v>482</v>
-      </c>
-      <c r="B103" t="s" s="2">
-        <v>482</v>
-      </c>
-      <c r="C103" s="2"/>
-      <c r="D103" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="E103" s="2"/>
-      <c r="F103" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="G103" t="s" s="2">
-        <v>42</v>
-      </c>
-      <c r="H103" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="I103" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="J103" t="s" s="2">
-        <v>43</v>
-      </c>
-      <c r="K103" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="L103" t="s" s="2">
-        <v>483</v>
-      </c>
-      <c r="M103" t="s" s="2">
-        <v>484</v>
-      </c>
-      <c r="N103" t="s" s="2">
-        <v>485</v>
-      </c>
-      <c r="O103" s="2"/>
-      <c r="P103" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Q103" s="2"/>
-      <c r="R103" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="S103" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="T103" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="U103" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="V103" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="W103" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="X103" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="Y103" t="s" s="2">
-        <v>486</v>
-      </c>
-      <c r="Z103" t="s" s="2">
-        <v>287</v>
-      </c>
-      <c r="AA103" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AB103" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AC103" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AD103" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AE103" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AF103" t="s" s="2">
-        <v>487</v>
-      </c>
-      <c r="AG103" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AH103" t="s" s="2">
-        <v>42</v>
-      </c>
-      <c r="AI103" t="s" s="2">
-        <v>54</v>
-      </c>
-      <c r="AJ103" t="s" s="2">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="104" hidden="true">
-      <c r="A104" t="s" s="2">
-        <v>488</v>
-      </c>
-      <c r="B104" t="s" s="2">
-        <v>488</v>
-      </c>
-      <c r="C104" s="2"/>
-      <c r="D104" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="E104" s="2"/>
-      <c r="F104" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="G104" t="s" s="2">
-        <v>42</v>
-      </c>
-      <c r="H104" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="I104" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="J104" t="s" s="2">
-        <v>43</v>
-      </c>
-      <c r="K104" t="s" s="2">
-        <v>215</v>
-      </c>
-      <c r="L104" t="s" s="2">
-        <v>489</v>
-      </c>
-      <c r="M104" t="s" s="2">
-        <v>490</v>
-      </c>
-      <c r="N104" t="s" s="2">
-        <v>491</v>
-      </c>
-      <c r="O104" s="2"/>
-      <c r="P104" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Q104" s="2"/>
-      <c r="R104" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="S104" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="T104" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="U104" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="V104" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="W104" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="X104" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Y104" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Z104" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AA104" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AB104" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AC104" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AD104" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AE104" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AF104" t="s" s="2">
-        <v>492</v>
-      </c>
-      <c r="AG104" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AH104" t="s" s="2">
-        <v>42</v>
-      </c>
-      <c r="AI104" t="s" s="2">
-        <v>54</v>
-      </c>
-      <c r="AJ104" t="s" s="2">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="105" hidden="true">
-      <c r="A105" t="s" s="2">
-        <v>493</v>
-      </c>
-      <c r="B105" t="s" s="2">
-        <v>493</v>
-      </c>
-      <c r="C105" s="2"/>
-      <c r="D105" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="E105" s="2"/>
-      <c r="F105" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="G105" t="s" s="2">
-        <v>42</v>
-      </c>
-      <c r="H105" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="I105" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="J105" t="s" s="2">
-        <v>43</v>
-      </c>
-      <c r="K105" t="s" s="2">
-        <v>56</v>
-      </c>
-      <c r="L105" t="s" s="2">
-        <v>494</v>
-      </c>
-      <c r="M105" t="s" s="2">
-        <v>495</v>
-      </c>
-      <c r="N105" t="s" s="2">
-        <v>496</v>
-      </c>
-      <c r="O105" s="2"/>
-      <c r="P105" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Q105" s="2"/>
-      <c r="R105" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="S105" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="T105" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="U105" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="V105" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="W105" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="X105" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Y105" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Z105" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AA105" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AB105" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AC105" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AD105" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AE105" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AF105" t="s" s="2">
-        <v>497</v>
-      </c>
-      <c r="AG105" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AH105" t="s" s="2">
-        <v>42</v>
-      </c>
-      <c r="AI105" t="s" s="2">
-        <v>54</v>
-      </c>
-      <c r="AJ105" t="s" s="2">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="106" hidden="true">
-      <c r="A106" t="s" s="2">
-        <v>498</v>
-      </c>
-      <c r="B106" t="s" s="2">
-        <v>498</v>
-      </c>
-      <c r="C106" s="2"/>
-      <c r="D106" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="E106" s="2"/>
-      <c r="F106" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="G106" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="H106" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="I106" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="J106" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="K106" t="s" s="2">
-        <v>499</v>
-      </c>
-      <c r="L106" t="s" s="2">
-        <v>500</v>
-      </c>
-      <c r="M106" t="s" s="2">
-        <v>501</v>
-      </c>
-      <c r="N106" t="s" s="2">
-        <v>502</v>
-      </c>
-      <c r="O106" t="s" s="2">
-        <v>503</v>
-      </c>
-      <c r="P106" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Q106" s="2"/>
-      <c r="R106" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="S106" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="T106" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="U106" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="V106" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="W106" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="X106" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Y106" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Z106" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AA106" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AB106" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AC106" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AD106" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AE106" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AF106" t="s" s="2">
-        <v>498</v>
-      </c>
-      <c r="AG106" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AH106" t="s" s="2">
-        <v>37</v>
-      </c>
-      <c r="AI106" t="s" s="2">
-        <v>54</v>
-      </c>
-      <c r="AJ106" t="s" s="2">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="107" hidden="true">
-      <c r="A107" t="s" s="2">
-        <v>504</v>
-      </c>
-      <c r="B107" t="s" s="2">
-        <v>504</v>
-      </c>
-      <c r="C107" s="2"/>
-      <c r="D107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="E107" s="2"/>
-      <c r="F107" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="G107" t="s" s="2">
-        <v>42</v>
-      </c>
-      <c r="H107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="I107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="J107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="K107" t="s" s="2">
-        <v>56</v>
-      </c>
-      <c r="L107" t="s" s="2">
-        <v>57</v>
-      </c>
-      <c r="M107" t="s" s="2">
-        <v>58</v>
-      </c>
-      <c r="N107" s="2"/>
-      <c r="O107" s="2"/>
-      <c r="P107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Q107" s="2"/>
-      <c r="R107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="S107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="T107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="U107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="V107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="W107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="X107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Y107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Z107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AA107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AB107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AC107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AD107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AE107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AF107" t="s" s="2">
-        <v>59</v>
-      </c>
-      <c r="AG107" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AH107" t="s" s="2">
-        <v>42</v>
-      </c>
-      <c r="AI107" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AJ107" t="s" s="2">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="108" hidden="true">
-      <c r="A108" t="s" s="2">
-        <v>505</v>
-      </c>
-      <c r="B108" t="s" s="2">
-        <v>505</v>
-      </c>
-      <c r="C108" s="2"/>
-      <c r="D108" t="s" s="2">
-        <v>61</v>
-      </c>
-      <c r="E108" s="2"/>
-      <c r="F108" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="G108" t="s" s="2">
-        <v>37</v>
-      </c>
-      <c r="H108" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="I108" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="J108" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="K108" t="s" s="2">
-        <v>62</v>
-      </c>
-      <c r="L108" t="s" s="2">
-        <v>63</v>
-      </c>
-      <c r="M108" t="s" s="2">
-        <v>64</v>
-      </c>
-      <c r="N108" t="s" s="2">
-        <v>65</v>
-      </c>
-      <c r="O108" s="2"/>
-      <c r="P108" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Q108" s="2"/>
-      <c r="R108" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="S108" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="T108" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="U108" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="V108" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="W108" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="X108" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Y108" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Z108" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AA108" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AB108" t="s" s="2">
-        <v>66</v>
-      </c>
-      <c r="AC108" t="s" s="2">
-        <v>67</v>
-      </c>
-      <c r="AD108" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AE108" t="s" s="2">
-        <v>68</v>
-      </c>
-      <c r="AF108" t="s" s="2">
-        <v>69</v>
-      </c>
-      <c r="AG108" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AH108" t="s" s="2">
-        <v>37</v>
-      </c>
-      <c r="AI108" t="s" s="2">
-        <v>54</v>
-      </c>
-      <c r="AJ108" t="s" s="2">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="109" hidden="true">
-      <c r="A109" t="s" s="2">
-        <v>506</v>
-      </c>
-      <c r="B109" t="s" s="2">
-        <v>506</v>
-      </c>
-      <c r="C109" s="2"/>
-      <c r="D109" t="s" s="2">
-        <v>507</v>
-      </c>
-      <c r="E109" s="2"/>
-      <c r="F109" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="G109" t="s" s="2">
-        <v>37</v>
-      </c>
-      <c r="H109" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="I109" t="s" s="2">
-        <v>43</v>
-      </c>
-      <c r="J109" t="s" s="2">
-        <v>43</v>
-      </c>
-      <c r="K109" t="s" s="2">
-        <v>62</v>
-      </c>
-      <c r="L109" t="s" s="2">
-        <v>508</v>
-      </c>
-      <c r="M109" t="s" s="2">
-        <v>509</v>
-      </c>
-      <c r="N109" t="s" s="2">
-        <v>65</v>
-      </c>
-      <c r="O109" t="s" s="2">
-        <v>212</v>
-      </c>
-      <c r="P109" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Q109" s="2"/>
-      <c r="R109" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="S109" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="T109" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="U109" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="V109" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="W109" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="X109" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Y109" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Z109" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AA109" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AB109" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AC109" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AD109" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AE109" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AF109" t="s" s="2">
-        <v>510</v>
-      </c>
-      <c r="AG109" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AH109" t="s" s="2">
-        <v>37</v>
-      </c>
-      <c r="AI109" t="s" s="2">
-        <v>54</v>
-      </c>
-      <c r="AJ109" t="s" s="2">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="110" hidden="true">
-      <c r="A110" t="s" s="2">
-        <v>511</v>
-      </c>
-      <c r="B110" t="s" s="2">
-        <v>511</v>
-      </c>
-      <c r="C110" s="2"/>
-      <c r="D110" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="E110" s="2"/>
-      <c r="F110" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="G110" t="s" s="2">
-        <v>42</v>
-      </c>
-      <c r="H110" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="I110" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="J110" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="K110" t="s" s="2">
-        <v>233</v>
-      </c>
-      <c r="L110" t="s" s="2">
-        <v>512</v>
-      </c>
-      <c r="M110" t="s" s="2">
-        <v>513</v>
-      </c>
-      <c r="N110" t="s" s="2">
-        <v>514</v>
-      </c>
-      <c r="O110" t="s" s="2">
-        <v>515</v>
-      </c>
-      <c r="P110" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Q110" s="2"/>
-      <c r="R110" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="S110" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="T110" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="U110" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="V110" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="W110" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="X110" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="Y110" t="s" s="2">
-        <v>516</v>
-      </c>
-      <c r="Z110" t="s" s="2">
-        <v>517</v>
-      </c>
-      <c r="AA110" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AB110" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AC110" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AD110" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AE110" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AF110" t="s" s="2">
-        <v>511</v>
-      </c>
-      <c r="AG110" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AH110" t="s" s="2">
-        <v>42</v>
-      </c>
-      <c r="AI110" t="s" s="2">
-        <v>54</v>
-      </c>
-      <c r="AJ110" t="s" s="2">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="111" hidden="true">
-      <c r="A111" t="s" s="2">
-        <v>518</v>
-      </c>
-      <c r="B111" t="s" s="2">
-        <v>518</v>
-      </c>
-      <c r="C111" s="2"/>
-      <c r="D111" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="E111" s="2"/>
-      <c r="F111" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="G111" t="s" s="2">
-        <v>42</v>
-      </c>
-      <c r="H111" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="I111" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="J111" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="K111" t="s" s="2">
-        <v>519</v>
-      </c>
-      <c r="L111" t="s" s="2">
-        <v>520</v>
-      </c>
-      <c r="M111" t="s" s="2">
-        <v>521</v>
-      </c>
-      <c r="N111" t="s" s="2">
-        <v>522</v>
-      </c>
-      <c r="O111" t="s" s="2">
-        <v>523</v>
-      </c>
-      <c r="P111" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Q111" s="2"/>
-      <c r="R111" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="S111" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="T111" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="U111" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="V111" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="W111" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="X111" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Y111" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Z111" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AA111" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AB111" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AC111" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AD111" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AE111" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AF111" t="s" s="2">
-        <v>518</v>
-      </c>
-      <c r="AG111" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AH111" t="s" s="2">
-        <v>42</v>
-      </c>
-      <c r="AI111" t="s" s="2">
-        <v>54</v>
-      </c>
-      <c r="AJ111" t="s" s="2">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="112" hidden="true">
-      <c r="A112" t="s" s="2">
-        <v>524</v>
-      </c>
-      <c r="B112" t="s" s="2">
-        <v>524</v>
-      </c>
-      <c r="C112" s="2"/>
-      <c r="D112" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="E112" s="2"/>
-      <c r="F112" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="G112" t="s" s="2">
-        <v>37</v>
-      </c>
-      <c r="H112" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="I112" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="J112" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="K112" t="s" s="2">
-        <v>404</v>
-      </c>
-      <c r="L112" t="s" s="2">
-        <v>460</v>
-      </c>
-      <c r="M112" t="s" s="2">
-        <v>406</v>
-      </c>
-      <c r="N112" s="2"/>
-      <c r="O112" t="s" s="2">
-        <v>525</v>
-      </c>
-      <c r="P112" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Q112" s="2"/>
-      <c r="R112" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="S112" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="T112" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="U112" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="V112" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="W112" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="X112" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Y112" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Z112" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AA112" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AB112" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AC112" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AD112" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AE112" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AF112" t="s" s="2">
-        <v>524</v>
-      </c>
-      <c r="AG112" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AH112" t="s" s="2">
-        <v>37</v>
-      </c>
-      <c r="AI112" t="s" s="2">
-        <v>54</v>
-      </c>
-      <c r="AJ112" t="s" s="2">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="113" hidden="true">
-      <c r="A113" t="s" s="2">
-        <v>527</v>
-      </c>
-      <c r="B113" t="s" s="2">
-        <v>527</v>
-      </c>
-      <c r="C113" s="2"/>
-      <c r="D113" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="E113" s="2"/>
-      <c r="F113" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="G113" t="s" s="2">
-        <v>42</v>
-      </c>
-      <c r="H113" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="I113" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="J113" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="K113" t="s" s="2">
-        <v>528</v>
-      </c>
-      <c r="L113" t="s" s="2">
-        <v>529</v>
-      </c>
-      <c r="M113" t="s" s="2">
-        <v>464</v>
-      </c>
-      <c r="N113" t="s" s="2">
-        <v>530</v>
-      </c>
-      <c r="O113" t="s" s="2">
-        <v>531</v>
-      </c>
-      <c r="P113" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Q113" s="2"/>
-      <c r="R113" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="S113" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="T113" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="U113" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="V113" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="W113" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="X113" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Y113" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Z113" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AA113" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AB113" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AC113" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AD113" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AE113" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AF113" t="s" s="2">
-        <v>527</v>
-      </c>
-      <c r="AG113" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AH113" t="s" s="2">
-        <v>42</v>
-      </c>
-      <c r="AI113" t="s" s="2">
-        <v>54</v>
-      </c>
-      <c r="AJ113" t="s" s="2">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="114" hidden="true">
-      <c r="A114" t="s" s="2">
-        <v>532</v>
-      </c>
-      <c r="B114" t="s" s="2">
-        <v>532</v>
-      </c>
-      <c r="C114" s="2"/>
-      <c r="D114" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="E114" s="2"/>
-      <c r="F114" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="G114" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="H114" t="s" s="2">
-        <v>43</v>
-      </c>
-      <c r="I114" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="J114" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="K114" t="s" s="2">
-        <v>533</v>
-      </c>
-      <c r="L114" t="s" s="2">
-        <v>534</v>
-      </c>
-      <c r="M114" t="s" s="2">
-        <v>535</v>
-      </c>
-      <c r="N114" t="s" s="2">
-        <v>536</v>
-      </c>
-      <c r="O114" t="s" s="2">
-        <v>537</v>
-      </c>
-      <c r="P114" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Q114" s="2"/>
-      <c r="R114" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="S114" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="T114" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="U114" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="V114" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="W114" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="X114" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Y114" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="Z114" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AA114" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AB114" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AC114" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AD114" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AE114" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="AF114" t="s" s="2">
-        <v>532</v>
-      </c>
-      <c r="AG114" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="AH114" t="s" s="2">
-        <v>37</v>
-      </c>
-      <c r="AI114" t="s" s="2">
-        <v>54</v>
-      </c>
-      <c r="AJ114" t="s" s="2">
         <v>267</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AJ114">
+  <autoFilter ref="A1:AJ102">
     <filterColumn colId="6">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -13768,7 +12401,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI113">
+  <conditionalFormatting sqref="A2:AI101">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>